<commit_message>
fix: harden task attachment validation
</commit_message>
<xml_diff>
--- a/tests/fixtures/media/workbook.xlsx
+++ b/tests/fixtures/media/workbook.xlsx
@@ -1,4 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<root/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheets/>
+</workbook>
 </file>
</xml_diff>